<commit_message>
Add Method C switch: V_ditch off for survey-only storage
Parametres B25=0 (default) uses SS_Amont volume only; Q_900+Q_overflow
unchanged. B25=1 restores trapezoid V_ditch. Original Ø900 file untouched.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
@@ -2024,6 +2024,21 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Inclure V_ditch trapèze? (1=oui, 0=levé seul)</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0 = recommandé si SS_Amont contient déjà le fossé (V=levé seul; Q_overflow garde b,z,L,n,S). 1 = ajoute V_ditch = A_trapèze × L (ancien mode — risque de double volume).</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
@@ -2107,7 +2122,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Longueur pour V_ditch = A × L et Manning</t>
+          <t>L pour Manning Q_overflow (et V_ditch seulement si B25=1)</t>
         </is>
       </c>
     </row>
@@ -2134,14 +2149,13 @@
           <t>Stockage_C (volume)</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>V_pond(levé) + V_ditch</t>
-        </is>
+      <c r="B34">
+        <f>IF(B25=1,"V_pond(levé)+V_ditch","V_pond(levé) seul")</f>
+        <v/>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Volume = bassin (levé) + fossé — Compose_900 + Calcul_C</t>
+          <t>Piloté par B25 — pas de double comptage si le fossé est déjà dans SS_Amont</t>
         </is>
       </c>
     </row>
@@ -2303,17 +2317,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Vmax_C (m³) = max(V_pond + V_ditch)</t>
+          <t>Vmax_C (m³) = max(V_total)</t>
         </is>
       </c>
       <c r="B49" s="20">
         <f>Calcul_C!B7</f>
         <v/>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Stockage total routé (levé + fossé)</t>
-        </is>
+      <c r="C49">
+        <f>IF(B25=1,"V_pond+V_ditch (B25=1)","V_pond seul — levé SS_Amont (B25=0)")</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -2431,7 +2444,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2) C (Zone 1): Qout = Q_900(WSE)+Q_overflow; V = V_pond(SS_Amont)+V_ditch; WSEmax_C = Calcul_C.</t>
+          <t>2) C (Zone 1): Qout = Q_900+Q_overflow; V = SS_Amont (+V_ditch si B25=1); WSEmax_C = Calcul_C.</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2549,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>• Méthode C: Qout = Q_900 + Q_overflow; V = V_pond + V_ditch — Compose_900 + Calcul_C (B49–B52).</t>
+          <t>• Méthode C: Qout = Q_900 + Q_overflow; V_ditch via B25 (0=levé seul) — Compose_900 + Calcul_C (B49–B52).</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3730,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   C) Qout = Q_900(WSE) + Q_overflow(WSE); V = V_pond + V_ditch → Compose_900 + Calcul_C.</t>
+          <t xml:space="preserve">   C) Qout = Q_900 + Q_overflow; V = V_pond (+ V_ditch si B25=1) → Compose_900 + Calcul_C.</t>
         </is>
       </c>
     </row>
@@ -7116,7 +7129,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Qout = Q_900(WSE) + Q_overflow(WSE). V_total = V_pond(SS_Amont) + V_ditch. Overflow: trapèze au-dessus du crown, Manning. Paramètres jaunes = Parametres!B27–B32.</t>
+          <t>Qout = Q_900(WSE) + Q_overflow(WSE). V_total = V_pond(SS_Amont) + (B25)*V_ditch. Qout = Q_900 + Q_overflow (trapèze Manning) toujours. B25=0 → pas de volume trapèze (levé seul). Paramètres = Parametres!B25–B32.</t>
         </is>
       </c>
     </row>
@@ -7205,6 +7218,17 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Inclure V_ditch (0/1)</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>Parametres!B25</f>
+        <v/>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -7279,7 +7303,7 @@
         <v/>
       </c>
       <c r="E15" s="26">
-        <f>D15*$B$11</f>
+        <f>IF($B$13=1,D15*$B$11,0)</f>
         <v/>
       </c>
       <c r="F15" s="26">
@@ -7287,7 +7311,7 @@
         <v/>
       </c>
       <c r="G15" s="34">
-        <f>E15+F15</f>
+        <f>F15+E15</f>
         <v/>
       </c>
       <c r="H15" s="5">
@@ -7324,7 +7348,7 @@
         <v/>
       </c>
       <c r="E16" s="26">
-        <f>D16*$B$11</f>
+        <f>IF($B$13=1,D16*$B$11,0)</f>
         <v/>
       </c>
       <c r="F16" s="26">
@@ -7332,7 +7356,7 @@
         <v/>
       </c>
       <c r="G16" s="34">
-        <f>E16+F16</f>
+        <f>F16+E16</f>
         <v/>
       </c>
       <c r="H16" s="5">
@@ -7369,7 +7393,7 @@
         <v/>
       </c>
       <c r="E17" s="26">
-        <f>D17*$B$11</f>
+        <f>IF($B$13=1,D17*$B$11,0)</f>
         <v/>
       </c>
       <c r="F17" s="26">
@@ -7377,7 +7401,7 @@
         <v/>
       </c>
       <c r="G17" s="34">
-        <f>E17+F17</f>
+        <f>F17+E17</f>
         <v/>
       </c>
       <c r="H17" s="5">
@@ -7414,7 +7438,7 @@
         <v/>
       </c>
       <c r="E18" s="26">
-        <f>D18*$B$11</f>
+        <f>IF($B$13=1,D18*$B$11,0)</f>
         <v/>
       </c>
       <c r="F18" s="26">
@@ -7422,7 +7446,7 @@
         <v/>
       </c>
       <c r="G18" s="34">
-        <f>E18+F18</f>
+        <f>F18+E18</f>
         <v/>
       </c>
       <c r="H18" s="5">
@@ -7459,7 +7483,7 @@
         <v/>
       </c>
       <c r="E19" s="26">
-        <f>D19*$B$11</f>
+        <f>IF($B$13=1,D19*$B$11,0)</f>
         <v/>
       </c>
       <c r="F19" s="26">
@@ -7467,7 +7491,7 @@
         <v/>
       </c>
       <c r="G19" s="34">
-        <f>E19+F19</f>
+        <f>F19+E19</f>
         <v/>
       </c>
       <c r="H19" s="5">
@@ -7504,7 +7528,7 @@
         <v/>
       </c>
       <c r="E20" s="26">
-        <f>D20*$B$11</f>
+        <f>IF($B$13=1,D20*$B$11,0)</f>
         <v/>
       </c>
       <c r="F20" s="26">
@@ -7512,7 +7536,7 @@
         <v/>
       </c>
       <c r="G20" s="34">
-        <f>E20+F20</f>
+        <f>F20+E20</f>
         <v/>
       </c>
       <c r="H20" s="5">
@@ -7549,7 +7573,7 @@
         <v/>
       </c>
       <c r="E21" s="26">
-        <f>D21*$B$11</f>
+        <f>IF($B$13=1,D21*$B$11,0)</f>
         <v/>
       </c>
       <c r="F21" s="26">
@@ -7557,7 +7581,7 @@
         <v/>
       </c>
       <c r="G21" s="34">
-        <f>E21+F21</f>
+        <f>F21+E21</f>
         <v/>
       </c>
       <c r="H21" s="5">
@@ -7594,7 +7618,7 @@
         <v/>
       </c>
       <c r="E22" s="26">
-        <f>D22*$B$11</f>
+        <f>IF($B$13=1,D22*$B$11,0)</f>
         <v/>
       </c>
       <c r="F22" s="26">
@@ -7602,7 +7626,7 @@
         <v/>
       </c>
       <c r="G22" s="34">
-        <f>E22+F22</f>
+        <f>F22+E22</f>
         <v/>
       </c>
       <c r="H22" s="5">
@@ -7639,7 +7663,7 @@
         <v/>
       </c>
       <c r="E23" s="26">
-        <f>D23*$B$11</f>
+        <f>IF($B$13=1,D23*$B$11,0)</f>
         <v/>
       </c>
       <c r="F23" s="26">
@@ -7647,7 +7671,7 @@
         <v/>
       </c>
       <c r="G23" s="34">
-        <f>E23+F23</f>
+        <f>F23+E23</f>
         <v/>
       </c>
       <c r="H23" s="5">
@@ -7684,7 +7708,7 @@
         <v/>
       </c>
       <c r="E24" s="26">
-        <f>D24*$B$11</f>
+        <f>IF($B$13=1,D24*$B$11,0)</f>
         <v/>
       </c>
       <c r="F24" s="26">
@@ -7692,7 +7716,7 @@
         <v/>
       </c>
       <c r="G24" s="34">
-        <f>E24+F24</f>
+        <f>F24+E24</f>
         <v/>
       </c>
       <c r="H24" s="5">
@@ -7729,7 +7753,7 @@
         <v/>
       </c>
       <c r="E25" s="26">
-        <f>D25*$B$11</f>
+        <f>IF($B$13=1,D25*$B$11,0)</f>
         <v/>
       </c>
       <c r="F25" s="26">
@@ -7737,7 +7761,7 @@
         <v/>
       </c>
       <c r="G25" s="34">
-        <f>E25+F25</f>
+        <f>F25+E25</f>
         <v/>
       </c>
       <c r="H25" s="5">
@@ -7774,7 +7798,7 @@
         <v/>
       </c>
       <c r="E26" s="26">
-        <f>D26*$B$11</f>
+        <f>IF($B$13=1,D26*$B$11,0)</f>
         <v/>
       </c>
       <c r="F26" s="26">
@@ -7782,7 +7806,7 @@
         <v/>
       </c>
       <c r="G26" s="34">
-        <f>E26+F26</f>
+        <f>F26+E26</f>
         <v/>
       </c>
       <c r="H26" s="5">
@@ -7819,7 +7843,7 @@
         <v/>
       </c>
       <c r="E27" s="26">
-        <f>D27*$B$11</f>
+        <f>IF($B$13=1,D27*$B$11,0)</f>
         <v/>
       </c>
       <c r="F27" s="26">
@@ -7827,7 +7851,7 @@
         <v/>
       </c>
       <c r="G27" s="34">
-        <f>E27+F27</f>
+        <f>F27+E27</f>
         <v/>
       </c>
       <c r="H27" s="5">
@@ -7864,7 +7888,7 @@
         <v/>
       </c>
       <c r="E28" s="26">
-        <f>D28*$B$11</f>
+        <f>IF($B$13=1,D28*$B$11,0)</f>
         <v/>
       </c>
       <c r="F28" s="26">
@@ -7872,7 +7896,7 @@
         <v/>
       </c>
       <c r="G28" s="34">
-        <f>E28+F28</f>
+        <f>F28+E28</f>
         <v/>
       </c>
       <c r="H28" s="5">
@@ -7909,7 +7933,7 @@
         <v/>
       </c>
       <c r="E29" s="26">
-        <f>D29*$B$11</f>
+        <f>IF($B$13=1,D29*$B$11,0)</f>
         <v/>
       </c>
       <c r="F29" s="26">
@@ -7917,7 +7941,7 @@
         <v/>
       </c>
       <c r="G29" s="34">
-        <f>E29+F29</f>
+        <f>F29+E29</f>
         <v/>
       </c>
       <c r="H29" s="5">
@@ -7954,7 +7978,7 @@
         <v/>
       </c>
       <c r="E30" s="26">
-        <f>D30*$B$11</f>
+        <f>IF($B$13=1,D30*$B$11,0)</f>
         <v/>
       </c>
       <c r="F30" s="26">
@@ -7962,7 +7986,7 @@
         <v/>
       </c>
       <c r="G30" s="34">
-        <f>E30+F30</f>
+        <f>F30+E30</f>
         <v/>
       </c>
       <c r="H30" s="5">
@@ -7999,7 +8023,7 @@
         <v/>
       </c>
       <c r="E31" s="26">
-        <f>D31*$B$11</f>
+        <f>IF($B$13=1,D31*$B$11,0)</f>
         <v/>
       </c>
       <c r="F31" s="26">
@@ -8007,7 +8031,7 @@
         <v/>
       </c>
       <c r="G31" s="34">
-        <f>E31+F31</f>
+        <f>F31+E31</f>
         <v/>
       </c>
       <c r="H31" s="5">
@@ -8044,7 +8068,7 @@
         <v/>
       </c>
       <c r="E32" s="26">
-        <f>D32*$B$11</f>
+        <f>IF($B$13=1,D32*$B$11,0)</f>
         <v/>
       </c>
       <c r="F32" s="26">
@@ -8052,7 +8076,7 @@
         <v/>
       </c>
       <c r="G32" s="34">
-        <f>E32+F32</f>
+        <f>F32+E32</f>
         <v/>
       </c>
       <c r="H32" s="5">
@@ -8089,7 +8113,7 @@
         <v/>
       </c>
       <c r="E33" s="42">
-        <f>D33*$B$11</f>
+        <f>IF($B$13=1,D33*$B$11,0)</f>
         <v/>
       </c>
       <c r="F33" s="42">
@@ -8097,7 +8121,7 @@
         <v/>
       </c>
       <c r="G33" s="34">
-        <f>E33+F33</f>
+        <f>F33+E33</f>
         <v/>
       </c>
       <c r="H33" s="8">
@@ -8134,7 +8158,7 @@
         <v/>
       </c>
       <c r="E34" s="26">
-        <f>D34*$B$11</f>
+        <f>IF($B$13=1,D34*$B$11,0)</f>
         <v/>
       </c>
       <c r="F34" s="26">
@@ -8142,7 +8166,7 @@
         <v/>
       </c>
       <c r="G34" s="34">
-        <f>E34+F34</f>
+        <f>F34+E34</f>
         <v/>
       </c>
       <c r="H34" s="5">
@@ -8179,7 +8203,7 @@
         <v/>
       </c>
       <c r="E35" s="26">
-        <f>D35*$B$11</f>
+        <f>IF($B$13=1,D35*$B$11,0)</f>
         <v/>
       </c>
       <c r="F35" s="26">
@@ -8187,7 +8211,7 @@
         <v/>
       </c>
       <c r="G35" s="34">
-        <f>E35+F35</f>
+        <f>F35+E35</f>
         <v/>
       </c>
       <c r="H35" s="5">
@@ -8224,7 +8248,7 @@
         <v/>
       </c>
       <c r="E36" s="26">
-        <f>D36*$B$11</f>
+        <f>IF($B$13=1,D36*$B$11,0)</f>
         <v/>
       </c>
       <c r="F36" s="26">
@@ -8232,7 +8256,7 @@
         <v/>
       </c>
       <c r="G36" s="34">
-        <f>E36+F36</f>
+        <f>F36+E36</f>
         <v/>
       </c>
       <c r="H36" s="5">
@@ -8269,7 +8293,7 @@
         <v/>
       </c>
       <c r="E37" s="26">
-        <f>D37*$B$11</f>
+        <f>IF($B$13=1,D37*$B$11,0)</f>
         <v/>
       </c>
       <c r="F37" s="26">
@@ -8277,7 +8301,7 @@
         <v/>
       </c>
       <c r="G37" s="34">
-        <f>E37+F37</f>
+        <f>F37+E37</f>
         <v/>
       </c>
       <c r="H37" s="5">
@@ -8314,7 +8338,7 @@
         <v/>
       </c>
       <c r="E38" s="26">
-        <f>D38*$B$11</f>
+        <f>IF($B$13=1,D38*$B$11,0)</f>
         <v/>
       </c>
       <c r="F38" s="26">
@@ -8322,7 +8346,7 @@
         <v/>
       </c>
       <c r="G38" s="34">
-        <f>E38+F38</f>
+        <f>F38+E38</f>
         <v/>
       </c>
       <c r="H38" s="5">
@@ -8359,7 +8383,7 @@
         <v/>
       </c>
       <c r="E39" s="26">
-        <f>D39*$B$11</f>
+        <f>IF($B$13=1,D39*$B$11,0)</f>
         <v/>
       </c>
       <c r="F39" s="26">
@@ -8367,7 +8391,7 @@
         <v/>
       </c>
       <c r="G39" s="34">
-        <f>E39+F39</f>
+        <f>F39+E39</f>
         <v/>
       </c>
       <c r="H39" s="5">
@@ -8404,7 +8428,7 @@
         <v/>
       </c>
       <c r="E40" s="26">
-        <f>D40*$B$11</f>
+        <f>IF($B$13=1,D40*$B$11,0)</f>
         <v/>
       </c>
       <c r="F40" s="26">
@@ -8412,7 +8436,7 @@
         <v/>
       </c>
       <c r="G40" s="34">
-        <f>E40+F40</f>
+        <f>F40+E40</f>
         <v/>
       </c>
       <c r="H40" s="5">
@@ -8449,7 +8473,7 @@
         <v/>
       </c>
       <c r="E41" s="26">
-        <f>D41*$B$11</f>
+        <f>IF($B$13=1,D41*$B$11,0)</f>
         <v/>
       </c>
       <c r="F41" s="26">
@@ -8457,7 +8481,7 @@
         <v/>
       </c>
       <c r="G41" s="34">
-        <f>E41+F41</f>
+        <f>F41+E41</f>
         <v/>
       </c>
       <c r="H41" s="5">
@@ -8494,7 +8518,7 @@
         <v/>
       </c>
       <c r="E42" s="26">
-        <f>D42*$B$11</f>
+        <f>IF($B$13=1,D42*$B$11,0)</f>
         <v/>
       </c>
       <c r="F42" s="26">
@@ -8502,7 +8526,7 @@
         <v/>
       </c>
       <c r="G42" s="34">
-        <f>E42+F42</f>
+        <f>F42+E42</f>
         <v/>
       </c>
       <c r="H42" s="5">
@@ -8539,7 +8563,7 @@
         <v/>
       </c>
       <c r="E43" s="26">
-        <f>D43*$B$11</f>
+        <f>IF($B$13=1,D43*$B$11,0)</f>
         <v/>
       </c>
       <c r="F43" s="26">
@@ -8547,7 +8571,7 @@
         <v/>
       </c>
       <c r="G43" s="34">
-        <f>E43+F43</f>
+        <f>F43+E43</f>
         <v/>
       </c>
       <c r="H43" s="5">
@@ -8584,7 +8608,7 @@
         <v/>
       </c>
       <c r="E44" s="26">
-        <f>D44*$B$11</f>
+        <f>IF($B$13=1,D44*$B$11,0)</f>
         <v/>
       </c>
       <c r="F44" s="26">
@@ -8592,7 +8616,7 @@
         <v/>
       </c>
       <c r="G44" s="34">
-        <f>E44+F44</f>
+        <f>F44+E44</f>
         <v/>
       </c>
       <c r="H44" s="5">
@@ -8629,7 +8653,7 @@
         <v/>
       </c>
       <c r="E45" s="26">
-        <f>D45*$B$11</f>
+        <f>IF($B$13=1,D45*$B$11,0)</f>
         <v/>
       </c>
       <c r="F45" s="26">
@@ -8637,7 +8661,7 @@
         <v/>
       </c>
       <c r="G45" s="34">
-        <f>E45+F45</f>
+        <f>F45+E45</f>
         <v/>
       </c>
       <c r="H45" s="5">
@@ -8674,7 +8698,7 @@
         <v/>
       </c>
       <c r="E46" s="26">
-        <f>D46*$B$11</f>
+        <f>IF($B$13=1,D46*$B$11,0)</f>
         <v/>
       </c>
       <c r="F46" s="26">
@@ -8682,7 +8706,7 @@
         <v/>
       </c>
       <c r="G46" s="34">
-        <f>E46+F46</f>
+        <f>F46+E46</f>
         <v/>
       </c>
       <c r="H46" s="5">
@@ -8719,7 +8743,7 @@
         <v/>
       </c>
       <c r="E47" s="26">
-        <f>D47*$B$11</f>
+        <f>IF($B$13=1,D47*$B$11,0)</f>
         <v/>
       </c>
       <c r="F47" s="26">
@@ -8727,7 +8751,7 @@
         <v/>
       </c>
       <c r="G47" s="34">
-        <f>E47+F47</f>
+        <f>F47+E47</f>
         <v/>
       </c>
       <c r="H47" s="5">
@@ -8764,7 +8788,7 @@
         <v/>
       </c>
       <c r="E48" s="26">
-        <f>D48*$B$11</f>
+        <f>IF($B$13=1,D48*$B$11,0)</f>
         <v/>
       </c>
       <c r="F48" s="26">
@@ -8772,7 +8796,7 @@
         <v/>
       </c>
       <c r="G48" s="34">
-        <f>E48+F48</f>
+        <f>F48+E48</f>
         <v/>
       </c>
       <c r="H48" s="5">
@@ -8809,7 +8833,7 @@
         <v/>
       </c>
       <c r="E49" s="26">
-        <f>D49*$B$11</f>
+        <f>IF($B$13=1,D49*$B$11,0)</f>
         <v/>
       </c>
       <c r="F49" s="26">
@@ -8817,7 +8841,7 @@
         <v/>
       </c>
       <c r="G49" s="34">
-        <f>E49+F49</f>
+        <f>F49+E49</f>
         <v/>
       </c>
       <c r="H49" s="5">
@@ -8854,7 +8878,7 @@
         <v/>
       </c>
       <c r="E50" s="26">
-        <f>D50*$B$11</f>
+        <f>IF($B$13=1,D50*$B$11,0)</f>
         <v/>
       </c>
       <c r="F50" s="26">
@@ -8862,7 +8886,7 @@
         <v/>
       </c>
       <c r="G50" s="34">
-        <f>E50+F50</f>
+        <f>F50+E50</f>
         <v/>
       </c>
       <c r="H50" s="5">
@@ -8899,7 +8923,7 @@
         <v/>
       </c>
       <c r="E51" s="26">
-        <f>D51*$B$11</f>
+        <f>IF($B$13=1,D51*$B$11,0)</f>
         <v/>
       </c>
       <c r="F51" s="26">
@@ -8907,7 +8931,7 @@
         <v/>
       </c>
       <c r="G51" s="34">
-        <f>E51+F51</f>
+        <f>F51+E51</f>
         <v/>
       </c>
       <c r="H51" s="5">
@@ -8944,7 +8968,7 @@
         <v/>
       </c>
       <c r="E52" s="26">
-        <f>D52*$B$11</f>
+        <f>IF($B$13=1,D52*$B$11,0)</f>
         <v/>
       </c>
       <c r="F52" s="26">
@@ -8952,7 +8976,7 @@
         <v/>
       </c>
       <c r="G52" s="34">
-        <f>E52+F52</f>
+        <f>F52+E52</f>
         <v/>
       </c>
       <c r="H52" s="5">
@@ -8989,7 +9013,7 @@
         <v/>
       </c>
       <c r="E53" s="26">
-        <f>D53*$B$11</f>
+        <f>IF($B$13=1,D53*$B$11,0)</f>
         <v/>
       </c>
       <c r="F53" s="26">
@@ -8997,7 +9021,7 @@
         <v/>
       </c>
       <c r="G53" s="34">
-        <f>E53+F53</f>
+        <f>F53+E53</f>
         <v/>
       </c>
       <c r="H53" s="5">
@@ -9034,7 +9058,7 @@
         <v/>
       </c>
       <c r="E54" s="26">
-        <f>D54*$B$11</f>
+        <f>IF($B$13=1,D54*$B$11,0)</f>
         <v/>
       </c>
       <c r="F54" s="26">
@@ -9042,7 +9066,7 @@
         <v/>
       </c>
       <c r="G54" s="34">
-        <f>E54+F54</f>
+        <f>F54+E54</f>
         <v/>
       </c>
       <c r="H54" s="5">
@@ -9079,7 +9103,7 @@
         <v/>
       </c>
       <c r="E55" s="26">
-        <f>D55*$B$11</f>
+        <f>IF($B$13=1,D55*$B$11,0)</f>
         <v/>
       </c>
       <c r="F55" s="26">
@@ -9087,7 +9111,7 @@
         <v/>
       </c>
       <c r="G55" s="34">
-        <f>E55+F55</f>
+        <f>F55+E55</f>
         <v/>
       </c>
       <c r="H55" s="5">
@@ -9124,7 +9148,7 @@
         <v/>
       </c>
       <c r="E56" s="26">
-        <f>D56*$B$11</f>
+        <f>IF($B$13=1,D56*$B$11,0)</f>
         <v/>
       </c>
       <c r="F56" s="26">
@@ -9132,7 +9156,7 @@
         <v/>
       </c>
       <c r="G56" s="34">
-        <f>E56+F56</f>
+        <f>F56+E56</f>
         <v/>
       </c>
       <c r="H56" s="5">
@@ -9169,7 +9193,7 @@
         <v/>
       </c>
       <c r="E57" s="26">
-        <f>D57*$B$11</f>
+        <f>IF($B$13=1,D57*$B$11,0)</f>
         <v/>
       </c>
       <c r="F57" s="26">
@@ -9177,7 +9201,7 @@
         <v/>
       </c>
       <c r="G57" s="34">
-        <f>E57+F57</f>
+        <f>F57+E57</f>
         <v/>
       </c>
       <c r="H57" s="5">
@@ -9214,7 +9238,7 @@
         <v/>
       </c>
       <c r="E58" s="26">
-        <f>D58*$B$11</f>
+        <f>IF($B$13=1,D58*$B$11,0)</f>
         <v/>
       </c>
       <c r="F58" s="26">
@@ -9222,7 +9246,7 @@
         <v/>
       </c>
       <c r="G58" s="34">
-        <f>E58+F58</f>
+        <f>F58+E58</f>
         <v/>
       </c>
       <c r="H58" s="5">
@@ -9259,7 +9283,7 @@
         <v/>
       </c>
       <c r="E59" s="26">
-        <f>D59*$B$11</f>
+        <f>IF($B$13=1,D59*$B$11,0)</f>
         <v/>
       </c>
       <c r="F59" s="26">
@@ -9267,7 +9291,7 @@
         <v/>
       </c>
       <c r="G59" s="34">
-        <f>E59+F59</f>
+        <f>F59+E59</f>
         <v/>
       </c>
       <c r="H59" s="5">
@@ -9304,7 +9328,7 @@
         <v/>
       </c>
       <c r="E60" s="26">
-        <f>D60*$B$11</f>
+        <f>IF($B$13=1,D60*$B$11,0)</f>
         <v/>
       </c>
       <c r="F60" s="26">
@@ -9312,7 +9336,7 @@
         <v/>
       </c>
       <c r="G60" s="34">
-        <f>E60+F60</f>
+        <f>F60+E60</f>
         <v/>
       </c>
       <c r="H60" s="5">
@@ -9349,7 +9373,7 @@
         <v/>
       </c>
       <c r="E61" s="26">
-        <f>D61*$B$11</f>
+        <f>IF($B$13=1,D61*$B$11,0)</f>
         <v/>
       </c>
       <c r="F61" s="26">
@@ -9357,7 +9381,7 @@
         <v/>
       </c>
       <c r="G61" s="34">
-        <f>E61+F61</f>
+        <f>F61+E61</f>
         <v/>
       </c>
       <c r="H61" s="5">
@@ -9394,7 +9418,7 @@
         <v/>
       </c>
       <c r="E62" s="26">
-        <f>D62*$B$11</f>
+        <f>IF($B$13=1,D62*$B$11,0)</f>
         <v/>
       </c>
       <c r="F62" s="26">
@@ -9402,7 +9426,7 @@
         <v/>
       </c>
       <c r="G62" s="34">
-        <f>E62+F62</f>
+        <f>F62+E62</f>
         <v/>
       </c>
       <c r="H62" s="5">
@@ -9439,7 +9463,7 @@
         <v/>
       </c>
       <c r="E63" s="26">
-        <f>D63*$B$11</f>
+        <f>IF($B$13=1,D63*$B$11,0)</f>
         <v/>
       </c>
       <c r="F63" s="26">
@@ -9447,7 +9471,7 @@
         <v/>
       </c>
       <c r="G63" s="34">
-        <f>E63+F63</f>
+        <f>F63+E63</f>
         <v/>
       </c>
       <c r="H63" s="5">
@@ -9484,7 +9508,7 @@
         <v/>
       </c>
       <c r="E64" s="26">
-        <f>D64*$B$11</f>
+        <f>IF($B$13=1,D64*$B$11,0)</f>
         <v/>
       </c>
       <c r="F64" s="26">
@@ -9492,7 +9516,7 @@
         <v/>
       </c>
       <c r="G64" s="34">
-        <f>E64+F64</f>
+        <f>F64+E64</f>
         <v/>
       </c>
       <c r="H64" s="5">
@@ -9529,7 +9553,7 @@
         <v/>
       </c>
       <c r="E65" s="26">
-        <f>D65*$B$11</f>
+        <f>IF($B$13=1,D65*$B$11,0)</f>
         <v/>
       </c>
       <c r="F65" s="26">
@@ -9537,7 +9561,7 @@
         <v/>
       </c>
       <c r="G65" s="34">
-        <f>E65+F65</f>
+        <f>F65+E65</f>
         <v/>
       </c>
       <c r="H65" s="5">
@@ -9574,7 +9598,7 @@
         <v/>
       </c>
       <c r="E66" s="26">
-        <f>D66*$B$11</f>
+        <f>IF($B$13=1,D66*$B$11,0)</f>
         <v/>
       </c>
       <c r="F66" s="26">
@@ -9582,7 +9606,7 @@
         <v/>
       </c>
       <c r="G66" s="34">
-        <f>E66+F66</f>
+        <f>F66+E66</f>
         <v/>
       </c>
       <c r="H66" s="5">
@@ -9619,7 +9643,7 @@
         <v/>
       </c>
       <c r="E67" s="26">
-        <f>D67*$B$11</f>
+        <f>IF($B$13=1,D67*$B$11,0)</f>
         <v/>
       </c>
       <c r="F67" s="26">
@@ -9627,7 +9651,7 @@
         <v/>
       </c>
       <c r="G67" s="34">
-        <f>E67+F67</f>
+        <f>F67+E67</f>
         <v/>
       </c>
       <c r="H67" s="5">
@@ -9664,7 +9688,7 @@
         <v/>
       </c>
       <c r="E68" s="26">
-        <f>D68*$B$11</f>
+        <f>IF($B$13=1,D68*$B$11,0)</f>
         <v/>
       </c>
       <c r="F68" s="26">
@@ -9672,7 +9696,7 @@
         <v/>
       </c>
       <c r="G68" s="34">
-        <f>E68+F68</f>
+        <f>F68+E68</f>
         <v/>
       </c>
       <c r="H68" s="5">
@@ -9709,7 +9733,7 @@
         <v/>
       </c>
       <c r="E69" s="26">
-        <f>D69*$B$11</f>
+        <f>IF($B$13=1,D69*$B$11,0)</f>
         <v/>
       </c>
       <c r="F69" s="26">
@@ -9717,7 +9741,7 @@
         <v/>
       </c>
       <c r="G69" s="34">
-        <f>E69+F69</f>
+        <f>F69+E69</f>
         <v/>
       </c>
       <c r="H69" s="5">
@@ -9754,7 +9778,7 @@
         <v/>
       </c>
       <c r="E70" s="26">
-        <f>D70*$B$11</f>
+        <f>IF($B$13=1,D70*$B$11,0)</f>
         <v/>
       </c>
       <c r="F70" s="26">
@@ -9762,7 +9786,7 @@
         <v/>
       </c>
       <c r="G70" s="34">
-        <f>E70+F70</f>
+        <f>F70+E70</f>
         <v/>
       </c>
       <c r="H70" s="5">
@@ -9799,7 +9823,7 @@
         <v/>
       </c>
       <c r="E71" s="26">
-        <f>D71*$B$11</f>
+        <f>IF($B$13=1,D71*$B$11,0)</f>
         <v/>
       </c>
       <c r="F71" s="26">
@@ -9807,7 +9831,7 @@
         <v/>
       </c>
       <c r="G71" s="34">
-        <f>E71+F71</f>
+        <f>F71+E71</f>
         <v/>
       </c>
       <c r="H71" s="5">
@@ -9844,7 +9868,7 @@
         <v/>
       </c>
       <c r="E72" s="26">
-        <f>D72*$B$11</f>
+        <f>IF($B$13=1,D72*$B$11,0)</f>
         <v/>
       </c>
       <c r="F72" s="26">
@@ -9852,7 +9876,7 @@
         <v/>
       </c>
       <c r="G72" s="34">
-        <f>E72+F72</f>
+        <f>F72+E72</f>
         <v/>
       </c>
       <c r="H72" s="5">
@@ -9889,7 +9913,7 @@
         <v/>
       </c>
       <c r="E73" s="26">
-        <f>D73*$B$11</f>
+        <f>IF($B$13=1,D73*$B$11,0)</f>
         <v/>
       </c>
       <c r="F73" s="26">
@@ -9897,7 +9921,7 @@
         <v/>
       </c>
       <c r="G73" s="34">
-        <f>E73+F73</f>
+        <f>F73+E73</f>
         <v/>
       </c>
       <c r="H73" s="5">
@@ -9934,7 +9958,7 @@
         <v/>
       </c>
       <c r="E74" s="26">
-        <f>D74*$B$11</f>
+        <f>IF($B$13=1,D74*$B$11,0)</f>
         <v/>
       </c>
       <c r="F74" s="26">
@@ -9942,7 +9966,7 @@
         <v/>
       </c>
       <c r="G74" s="34">
-        <f>E74+F74</f>
+        <f>F74+E74</f>
         <v/>
       </c>
       <c r="H74" s="5">
@@ -9979,7 +10003,7 @@
         <v/>
       </c>
       <c r="E75" s="26">
-        <f>D75*$B$11</f>
+        <f>IF($B$13=1,D75*$B$11,0)</f>
         <v/>
       </c>
       <c r="F75" s="26">
@@ -9987,7 +10011,7 @@
         <v/>
       </c>
       <c r="G75" s="34">
-        <f>E75+F75</f>
+        <f>F75+E75</f>
         <v/>
       </c>
       <c r="H75" s="5">
@@ -10024,7 +10048,7 @@
         <v/>
       </c>
       <c r="E76" s="26">
-        <f>D76*$B$11</f>
+        <f>IF($B$13=1,D76*$B$11,0)</f>
         <v/>
       </c>
       <c r="F76" s="26">
@@ -10032,7 +10056,7 @@
         <v/>
       </c>
       <c r="G76" s="34">
-        <f>E76+F76</f>
+        <f>F76+E76</f>
         <v/>
       </c>
       <c r="H76" s="5">
@@ -10069,7 +10093,7 @@
         <v/>
       </c>
       <c r="E77" s="26">
-        <f>D77*$B$11</f>
+        <f>IF($B$13=1,D77*$B$11,0)</f>
         <v/>
       </c>
       <c r="F77" s="26">
@@ -10077,7 +10101,7 @@
         <v/>
       </c>
       <c r="G77" s="34">
-        <f>E77+F77</f>
+        <f>F77+E77</f>
         <v/>
       </c>
       <c r="H77" s="5">
@@ -10114,7 +10138,7 @@
         <v/>
       </c>
       <c r="E78" s="26">
-        <f>D78*$B$11</f>
+        <f>IF($B$13=1,D78*$B$11,0)</f>
         <v/>
       </c>
       <c r="F78" s="26">
@@ -10122,7 +10146,7 @@
         <v/>
       </c>
       <c r="G78" s="34">
-        <f>E78+F78</f>
+        <f>F78+E78</f>
         <v/>
       </c>
       <c r="H78" s="5">
@@ -10159,7 +10183,7 @@
         <v/>
       </c>
       <c r="E79" s="26">
-        <f>D79*$B$11</f>
+        <f>IF($B$13=1,D79*$B$11,0)</f>
         <v/>
       </c>
       <c r="F79" s="26">
@@ -10167,7 +10191,7 @@
         <v/>
       </c>
       <c r="G79" s="34">
-        <f>E79+F79</f>
+        <f>F79+E79</f>
         <v/>
       </c>
       <c r="H79" s="5">
@@ -10204,7 +10228,7 @@
         <v/>
       </c>
       <c r="E80" s="26">
-        <f>D80*$B$11</f>
+        <f>IF($B$13=1,D80*$B$11,0)</f>
         <v/>
       </c>
       <c r="F80" s="26">
@@ -10212,7 +10236,7 @@
         <v/>
       </c>
       <c r="G80" s="34">
-        <f>E80+F80</f>
+        <f>F80+E80</f>
         <v/>
       </c>
       <c r="H80" s="5">
@@ -10249,7 +10273,7 @@
         <v/>
       </c>
       <c r="E81" s="26">
-        <f>D81*$B$11</f>
+        <f>IF($B$13=1,D81*$B$11,0)</f>
         <v/>
       </c>
       <c r="F81" s="26">
@@ -10257,7 +10281,7 @@
         <v/>
       </c>
       <c r="G81" s="34">
-        <f>E81+F81</f>
+        <f>F81+E81</f>
         <v/>
       </c>
       <c r="H81" s="5">
@@ -10294,7 +10318,7 @@
         <v/>
       </c>
       <c r="E82" s="26">
-        <f>D82*$B$11</f>
+        <f>IF($B$13=1,D82*$B$11,0)</f>
         <v/>
       </c>
       <c r="F82" s="26">
@@ -10302,7 +10326,7 @@
         <v/>
       </c>
       <c r="G82" s="34">
-        <f>E82+F82</f>
+        <f>F82+E82</f>
         <v/>
       </c>
       <c r="H82" s="5">
@@ -10339,7 +10363,7 @@
         <v/>
       </c>
       <c r="E83" s="26">
-        <f>D83*$B$11</f>
+        <f>IF($B$13=1,D83*$B$11,0)</f>
         <v/>
       </c>
       <c r="F83" s="26">
@@ -10347,7 +10371,7 @@
         <v/>
       </c>
       <c r="G83" s="34">
-        <f>E83+F83</f>
+        <f>F83+E83</f>
         <v/>
       </c>
       <c r="H83" s="5">
@@ -10384,7 +10408,7 @@
         <v/>
       </c>
       <c r="E84" s="26">
-        <f>D84*$B$11</f>
+        <f>IF($B$13=1,D84*$B$11,0)</f>
         <v/>
       </c>
       <c r="F84" s="26">
@@ -10392,7 +10416,7 @@
         <v/>
       </c>
       <c r="G84" s="34">
-        <f>E84+F84</f>
+        <f>F84+E84</f>
         <v/>
       </c>
       <c r="H84" s="5">
@@ -10429,7 +10453,7 @@
         <v/>
       </c>
       <c r="E85" s="26">
-        <f>D85*$B$11</f>
+        <f>IF($B$13=1,D85*$B$11,0)</f>
         <v/>
       </c>
       <c r="F85" s="26">
@@ -10437,7 +10461,7 @@
         <v/>
       </c>
       <c r="G85" s="34">
-        <f>E85+F85</f>
+        <f>F85+E85</f>
         <v/>
       </c>
       <c r="H85" s="5">
@@ -10474,7 +10498,7 @@
         <v/>
       </c>
       <c r="E86" s="26">
-        <f>D86*$B$11</f>
+        <f>IF($B$13=1,D86*$B$11,0)</f>
         <v/>
       </c>
       <c r="F86" s="26">
@@ -10482,7 +10506,7 @@
         <v/>
       </c>
       <c r="G86" s="34">
-        <f>E86+F86</f>
+        <f>F86+E86</f>
         <v/>
       </c>
       <c r="H86" s="5">
@@ -10519,7 +10543,7 @@
         <v/>
       </c>
       <c r="E87" s="26">
-        <f>D87*$B$11</f>
+        <f>IF($B$13=1,D87*$B$11,0)</f>
         <v/>
       </c>
       <c r="F87" s="26">
@@ -10527,7 +10551,7 @@
         <v/>
       </c>
       <c r="G87" s="34">
-        <f>E87+F87</f>
+        <f>F87+E87</f>
         <v/>
       </c>
       <c r="H87" s="5">
@@ -10564,7 +10588,7 @@
         <v/>
       </c>
       <c r="E88" s="26">
-        <f>D88*$B$11</f>
+        <f>IF($B$13=1,D88*$B$11,0)</f>
         <v/>
       </c>
       <c r="F88" s="26">
@@ -10572,7 +10596,7 @@
         <v/>
       </c>
       <c r="G88" s="34">
-        <f>E88+F88</f>
+        <f>F88+E88</f>
         <v/>
       </c>
       <c r="H88" s="5">
@@ -10609,7 +10633,7 @@
         <v/>
       </c>
       <c r="E89" s="26">
-        <f>D89*$B$11</f>
+        <f>IF($B$13=1,D89*$B$11,0)</f>
         <v/>
       </c>
       <c r="F89" s="26">
@@ -10617,7 +10641,7 @@
         <v/>
       </c>
       <c r="G89" s="34">
-        <f>E89+F89</f>
+        <f>F89+E89</f>
         <v/>
       </c>
       <c r="H89" s="5">
@@ -10654,7 +10678,7 @@
         <v/>
       </c>
       <c r="E90" s="26">
-        <f>D90*$B$11</f>
+        <f>IF($B$13=1,D90*$B$11,0)</f>
         <v/>
       </c>
       <c r="F90" s="26">
@@ -10662,7 +10686,7 @@
         <v/>
       </c>
       <c r="G90" s="34">
-        <f>E90+F90</f>
+        <f>F90+E90</f>
         <v/>
       </c>
       <c r="H90" s="5">
@@ -10699,7 +10723,7 @@
         <v/>
       </c>
       <c r="E91" s="26">
-        <f>D91*$B$11</f>
+        <f>IF($B$13=1,D91*$B$11,0)</f>
         <v/>
       </c>
       <c r="F91" s="26">
@@ -10707,7 +10731,7 @@
         <v/>
       </c>
       <c r="G91" s="34">
-        <f>E91+F91</f>
+        <f>F91+E91</f>
         <v/>
       </c>
       <c r="H91" s="5">
@@ -10744,7 +10768,7 @@
         <v/>
       </c>
       <c r="E92" s="26">
-        <f>D92*$B$11</f>
+        <f>IF($B$13=1,D92*$B$11,0)</f>
         <v/>
       </c>
       <c r="F92" s="26">
@@ -10752,7 +10776,7 @@
         <v/>
       </c>
       <c r="G92" s="34">
-        <f>E92+F92</f>
+        <f>F92+E92</f>
         <v/>
       </c>
       <c r="H92" s="5">
@@ -10789,7 +10813,7 @@
         <v/>
       </c>
       <c r="E93" s="26">
-        <f>D93*$B$11</f>
+        <f>IF($B$13=1,D93*$B$11,0)</f>
         <v/>
       </c>
       <c r="F93" s="26">
@@ -10797,7 +10821,7 @@
         <v/>
       </c>
       <c r="G93" s="34">
-        <f>E93+F93</f>
+        <f>F93+E93</f>
         <v/>
       </c>
       <c r="H93" s="5">
@@ -10834,7 +10858,7 @@
         <v/>
       </c>
       <c r="E94" s="26">
-        <f>D94*$B$11</f>
+        <f>IF($B$13=1,D94*$B$11,0)</f>
         <v/>
       </c>
       <c r="F94" s="26">
@@ -10842,7 +10866,7 @@
         <v/>
       </c>
       <c r="G94" s="34">
-        <f>E94+F94</f>
+        <f>F94+E94</f>
         <v/>
       </c>
       <c r="H94" s="5">
@@ -10879,7 +10903,7 @@
         <v/>
       </c>
       <c r="E95" s="26">
-        <f>D95*$B$11</f>
+        <f>IF($B$13=1,D95*$B$11,0)</f>
         <v/>
       </c>
       <c r="F95" s="26">
@@ -10887,7 +10911,7 @@
         <v/>
       </c>
       <c r="G95" s="34">
-        <f>E95+F95</f>
+        <f>F95+E95</f>
         <v/>
       </c>
       <c r="H95" s="5">
@@ -10924,7 +10948,7 @@
         <v/>
       </c>
       <c r="E96" s="26">
-        <f>D96*$B$11</f>
+        <f>IF($B$13=1,D96*$B$11,0)</f>
         <v/>
       </c>
       <c r="F96" s="26">
@@ -10932,7 +10956,7 @@
         <v/>
       </c>
       <c r="G96" s="34">
-        <f>E96+F96</f>
+        <f>F96+E96</f>
         <v/>
       </c>
       <c r="H96" s="5">
@@ -10969,7 +10993,7 @@
         <v/>
       </c>
       <c r="E97" s="26">
-        <f>D97*$B$11</f>
+        <f>IF($B$13=1,D97*$B$11,0)</f>
         <v/>
       </c>
       <c r="F97" s="26">
@@ -10977,7 +11001,7 @@
         <v/>
       </c>
       <c r="G97" s="34">
-        <f>E97+F97</f>
+        <f>F97+E97</f>
         <v/>
       </c>
       <c r="H97" s="5">
@@ -11014,7 +11038,7 @@
         <v/>
       </c>
       <c r="E98" s="26">
-        <f>D98*$B$11</f>
+        <f>IF($B$13=1,D98*$B$11,0)</f>
         <v/>
       </c>
       <c r="F98" s="26">
@@ -11022,7 +11046,7 @@
         <v/>
       </c>
       <c r="G98" s="34">
-        <f>E98+F98</f>
+        <f>F98+E98</f>
         <v/>
       </c>
       <c r="H98" s="5">
@@ -11059,7 +11083,7 @@
         <v/>
       </c>
       <c r="E99" s="26">
-        <f>D99*$B$11</f>
+        <f>IF($B$13=1,D99*$B$11,0)</f>
         <v/>
       </c>
       <c r="F99" s="26">
@@ -11067,7 +11091,7 @@
         <v/>
       </c>
       <c r="G99" s="34">
-        <f>E99+F99</f>
+        <f>F99+E99</f>
         <v/>
       </c>
       <c r="H99" s="5">
@@ -11104,7 +11128,7 @@
         <v/>
       </c>
       <c r="E100" s="26">
-        <f>D100*$B$11</f>
+        <f>IF($B$13=1,D100*$B$11,0)</f>
         <v/>
       </c>
       <c r="F100" s="26">
@@ -11112,7 +11136,7 @@
         <v/>
       </c>
       <c r="G100" s="34">
-        <f>E100+F100</f>
+        <f>F100+E100</f>
         <v/>
       </c>
       <c r="H100" s="5">
@@ -11149,7 +11173,7 @@
         <v/>
       </c>
       <c r="E101" s="26">
-        <f>D101*$B$11</f>
+        <f>IF($B$13=1,D101*$B$11,0)</f>
         <v/>
       </c>
       <c r="F101" s="26">
@@ -11157,7 +11181,7 @@
         <v/>
       </c>
       <c r="G101" s="34">
-        <f>E101+F101</f>
+        <f>F101+E101</f>
         <v/>
       </c>
       <c r="H101" s="5">
@@ -11194,7 +11218,7 @@
         <v/>
       </c>
       <c r="E102" s="26">
-        <f>D102*$B$11</f>
+        <f>IF($B$13=1,D102*$B$11,0)</f>
         <v/>
       </c>
       <c r="F102" s="26">
@@ -11202,7 +11226,7 @@
         <v/>
       </c>
       <c r="G102" s="34">
-        <f>E102+F102</f>
+        <f>F102+E102</f>
         <v/>
       </c>
       <c r="H102" s="5">
@@ -11239,7 +11263,7 @@
         <v/>
       </c>
       <c r="E103" s="26">
-        <f>D103*$B$11</f>
+        <f>IF($B$13=1,D103*$B$11,0)</f>
         <v/>
       </c>
       <c r="F103" s="26">
@@ -11247,7 +11271,7 @@
         <v/>
       </c>
       <c r="G103" s="34">
-        <f>E103+F103</f>
+        <f>F103+E103</f>
         <v/>
       </c>
       <c r="H103" s="5">
@@ -11284,7 +11308,7 @@
         <v/>
       </c>
       <c r="E104" s="26">
-        <f>D104*$B$11</f>
+        <f>IF($B$13=1,D104*$B$11,0)</f>
         <v/>
       </c>
       <c r="F104" s="26">
@@ -11292,7 +11316,7 @@
         <v/>
       </c>
       <c r="G104" s="34">
-        <f>E104+F104</f>
+        <f>F104+E104</f>
         <v/>
       </c>
       <c r="H104" s="5">
@@ -11329,7 +11353,7 @@
         <v/>
       </c>
       <c r="E105" s="26">
-        <f>D105*$B$11</f>
+        <f>IF($B$13=1,D105*$B$11,0)</f>
         <v/>
       </c>
       <c r="F105" s="26">
@@ -11337,7 +11361,7 @@
         <v/>
       </c>
       <c r="G105" s="34">
-        <f>E105+F105</f>
+        <f>F105+E105</f>
         <v/>
       </c>
       <c r="H105" s="5">
@@ -11374,7 +11398,7 @@
         <v/>
       </c>
       <c r="E106" s="26">
-        <f>D106*$B$11</f>
+        <f>IF($B$13=1,D106*$B$11,0)</f>
         <v/>
       </c>
       <c r="F106" s="26">
@@ -11382,7 +11406,7 @@
         <v/>
       </c>
       <c r="G106" s="34">
-        <f>E106+F106</f>
+        <f>F106+E106</f>
         <v/>
       </c>
       <c r="H106" s="5">
@@ -11419,7 +11443,7 @@
         <v/>
       </c>
       <c r="E107" s="26">
-        <f>D107*$B$11</f>
+        <f>IF($B$13=1,D107*$B$11,0)</f>
         <v/>
       </c>
       <c r="F107" s="26">
@@ -11427,7 +11451,7 @@
         <v/>
       </c>
       <c r="G107" s="34">
-        <f>E107+F107</f>
+        <f>F107+E107</f>
         <v/>
       </c>
       <c r="H107" s="5">
@@ -11477,14 +11501,14 @@
     <row r="1">
       <c r="A1" s="24" t="inlineStr">
         <is>
-          <t>Méthode C — routage avec Qout composé + V = V_pond + V_ditch</t>
+          <t>Méthode C — routage Qout composé; V = V_total (B25 pilote V_ditch)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>À chaque pas: WSE lu sur Compose_900!V_total → Qout sur Compose_900. ΔV = (Qin_moy − Qout)×Δt. Si V≈0, Qout = MIN(Qin, Q_plein).</t>
+          <t>À chaque pas: WSE lu sur Compose_900!V_total → Qout sur Compose_900. V_total = V_pond + V_ditch seulement si Parametres!B25=1; sinon V=levé SS_Amont. Q_overflow reste actif (b,z,L,n,S). ΔV = (Qin_moy − Qout)×Δt.</t>
         </is>
       </c>
     </row>
@@ -12332,10 +12356,9 @@
         <f>Parametres!B51</f>
         <v/>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Vmax_C inclut V_ditch</t>
-        </is>
+      <c r="D26">
+        <f>IF(Parametres!B25=1,"Vmax_C inclut V_ditch","Vmax_C = levé seul (B25=0)")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix unphysical velocities when overflow is active
Do not divide total Qout (pipe+overflow) by pipe area. Blank V_pipe when
WSE>crest; blank V_overflow for tiny ditch area; point users to Compose.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
@@ -1704,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2734,11 +2734,20 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="25" t="inlineStr">
+        <is>
+          <t>ATTENTION: des V &gt;&gt; 5–6 m/s ne sont PAS physiques. Souvent Q_overflow+Q_pipe divisé par A_tuyau, ou Q/A_fossé trop petit. Vitesses tuyau réalistes typ. ~1–4 m/s; lire Compose_900 (V_Ø900) et Courbe_QH_900.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92"/>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A91:H92"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A61:H61"/>
@@ -8254,7 +8263,7 @@
         <v/>
       </c>
       <c r="M15" s="27">
-        <f>IF(D15&lt;=0,0,I15/D15)</f>
+        <f>IF(OR(C15&lt;0.05,D15&lt;0.05),"",I15/D15)</f>
         <v/>
       </c>
     </row>
@@ -8307,7 +8316,7 @@
         <v/>
       </c>
       <c r="M16" s="27">
-        <f>IF(D16&lt;=0,0,I16/D16)</f>
+        <f>IF(OR(C16&lt;0.05,D16&lt;0.05),"",I16/D16)</f>
         <v/>
       </c>
     </row>
@@ -8360,7 +8369,7 @@
         <v/>
       </c>
       <c r="M17" s="27">
-        <f>IF(D17&lt;=0,0,I17/D17)</f>
+        <f>IF(OR(C17&lt;0.05,D17&lt;0.05),"",I17/D17)</f>
         <v/>
       </c>
     </row>
@@ -8413,7 +8422,7 @@
         <v/>
       </c>
       <c r="M18" s="27">
-        <f>IF(D18&lt;=0,0,I18/D18)</f>
+        <f>IF(OR(C18&lt;0.05,D18&lt;0.05),"",I18/D18)</f>
         <v/>
       </c>
     </row>
@@ -8466,7 +8475,7 @@
         <v/>
       </c>
       <c r="M19" s="27">
-        <f>IF(D19&lt;=0,0,I19/D19)</f>
+        <f>IF(OR(C19&lt;0.05,D19&lt;0.05),"",I19/D19)</f>
         <v/>
       </c>
     </row>
@@ -8519,7 +8528,7 @@
         <v/>
       </c>
       <c r="M20" s="27">
-        <f>IF(D20&lt;=0,0,I20/D20)</f>
+        <f>IF(OR(C20&lt;0.05,D20&lt;0.05),"",I20/D20)</f>
         <v/>
       </c>
     </row>
@@ -8572,7 +8581,7 @@
         <v/>
       </c>
       <c r="M21" s="27">
-        <f>IF(D21&lt;=0,0,I21/D21)</f>
+        <f>IF(OR(C21&lt;0.05,D21&lt;0.05),"",I21/D21)</f>
         <v/>
       </c>
     </row>
@@ -8625,7 +8634,7 @@
         <v/>
       </c>
       <c r="M22" s="27">
-        <f>IF(D22&lt;=0,0,I22/D22)</f>
+        <f>IF(OR(C22&lt;0.05,D22&lt;0.05),"",I22/D22)</f>
         <v/>
       </c>
     </row>
@@ -8678,7 +8687,7 @@
         <v/>
       </c>
       <c r="M23" s="27">
-        <f>IF(D23&lt;=0,0,I23/D23)</f>
+        <f>IF(OR(C23&lt;0.05,D23&lt;0.05),"",I23/D23)</f>
         <v/>
       </c>
     </row>
@@ -8731,7 +8740,7 @@
         <v/>
       </c>
       <c r="M24" s="27">
-        <f>IF(D24&lt;=0,0,I24/D24)</f>
+        <f>IF(OR(C24&lt;0.05,D24&lt;0.05),"",I24/D24)</f>
         <v/>
       </c>
     </row>
@@ -8784,7 +8793,7 @@
         <v/>
       </c>
       <c r="M25" s="27">
-        <f>IF(D25&lt;=0,0,I25/D25)</f>
+        <f>IF(OR(C25&lt;0.05,D25&lt;0.05),"",I25/D25)</f>
         <v/>
       </c>
     </row>
@@ -8837,7 +8846,7 @@
         <v/>
       </c>
       <c r="M26" s="27">
-        <f>IF(D26&lt;=0,0,I26/D26)</f>
+        <f>IF(OR(C26&lt;0.05,D26&lt;0.05),"",I26/D26)</f>
         <v/>
       </c>
     </row>
@@ -8890,7 +8899,7 @@
         <v/>
       </c>
       <c r="M27" s="27">
-        <f>IF(D27&lt;=0,0,I27/D27)</f>
+        <f>IF(OR(C27&lt;0.05,D27&lt;0.05),"",I27/D27)</f>
         <v/>
       </c>
     </row>
@@ -8943,7 +8952,7 @@
         <v/>
       </c>
       <c r="M28" s="27">
-        <f>IF(D28&lt;=0,0,I28/D28)</f>
+        <f>IF(OR(C28&lt;0.05,D28&lt;0.05),"",I28/D28)</f>
         <v/>
       </c>
     </row>
@@ -8996,7 +9005,7 @@
         <v/>
       </c>
       <c r="M29" s="27">
-        <f>IF(D29&lt;=0,0,I29/D29)</f>
+        <f>IF(OR(C29&lt;0.05,D29&lt;0.05),"",I29/D29)</f>
         <v/>
       </c>
     </row>
@@ -9049,7 +9058,7 @@
         <v/>
       </c>
       <c r="M30" s="27">
-        <f>IF(D30&lt;=0,0,I30/D30)</f>
+        <f>IF(OR(C30&lt;0.05,D30&lt;0.05),"",I30/D30)</f>
         <v/>
       </c>
     </row>
@@ -9102,7 +9111,7 @@
         <v/>
       </c>
       <c r="M31" s="27">
-        <f>IF(D31&lt;=0,0,I31/D31)</f>
+        <f>IF(OR(C31&lt;0.05,D31&lt;0.05),"",I31/D31)</f>
         <v/>
       </c>
     </row>
@@ -9155,7 +9164,7 @@
         <v/>
       </c>
       <c r="M32" s="27">
-        <f>IF(D32&lt;=0,0,I32/D32)</f>
+        <f>IF(OR(C32&lt;0.05,D32&lt;0.05),"",I32/D32)</f>
         <v/>
       </c>
     </row>
@@ -9208,7 +9217,7 @@
         <v/>
       </c>
       <c r="M33" s="27">
-        <f>IF(D33&lt;=0,0,I33/D33)</f>
+        <f>IF(OR(C33&lt;0.05,D33&lt;0.05),"",I33/D33)</f>
         <v/>
       </c>
     </row>
@@ -9261,7 +9270,7 @@
         <v/>
       </c>
       <c r="M34" s="27">
-        <f>IF(D34&lt;=0,0,I34/D34)</f>
+        <f>IF(OR(C34&lt;0.05,D34&lt;0.05),"",I34/D34)</f>
         <v/>
       </c>
     </row>
@@ -9314,7 +9323,7 @@
         <v/>
       </c>
       <c r="M35" s="27">
-        <f>IF(D35&lt;=0,0,I35/D35)</f>
+        <f>IF(OR(C35&lt;0.05,D35&lt;0.05),"",I35/D35)</f>
         <v/>
       </c>
     </row>
@@ -9367,7 +9376,7 @@
         <v/>
       </c>
       <c r="M36" s="27">
-        <f>IF(D36&lt;=0,0,I36/D36)</f>
+        <f>IF(OR(C36&lt;0.05,D36&lt;0.05),"",I36/D36)</f>
         <v/>
       </c>
     </row>
@@ -9420,7 +9429,7 @@
         <v/>
       </c>
       <c r="M37" s="27">
-        <f>IF(D37&lt;=0,0,I37/D37)</f>
+        <f>IF(OR(C37&lt;0.05,D37&lt;0.05),"",I37/D37)</f>
         <v/>
       </c>
     </row>
@@ -9473,7 +9482,7 @@
         <v/>
       </c>
       <c r="M38" s="27">
-        <f>IF(D38&lt;=0,0,I38/D38)</f>
+        <f>IF(OR(C38&lt;0.05,D38&lt;0.05),"",I38/D38)</f>
         <v/>
       </c>
     </row>
@@ -9526,7 +9535,7 @@
         <v/>
       </c>
       <c r="M39" s="27">
-        <f>IF(D39&lt;=0,0,I39/D39)</f>
+        <f>IF(OR(C39&lt;0.05,D39&lt;0.05),"",I39/D39)</f>
         <v/>
       </c>
     </row>
@@ -9579,7 +9588,7 @@
         <v/>
       </c>
       <c r="M40" s="27">
-        <f>IF(D40&lt;=0,0,I40/D40)</f>
+        <f>IF(OR(C40&lt;0.05,D40&lt;0.05),"",I40/D40)</f>
         <v/>
       </c>
     </row>
@@ -9632,7 +9641,7 @@
         <v/>
       </c>
       <c r="M41" s="27">
-        <f>IF(D41&lt;=0,0,I41/D41)</f>
+        <f>IF(OR(C41&lt;0.05,D41&lt;0.05),"",I41/D41)</f>
         <v/>
       </c>
     </row>
@@ -9685,7 +9694,7 @@
         <v/>
       </c>
       <c r="M42" s="27">
-        <f>IF(D42&lt;=0,0,I42/D42)</f>
+        <f>IF(OR(C42&lt;0.05,D42&lt;0.05),"",I42/D42)</f>
         <v/>
       </c>
     </row>
@@ -9738,7 +9747,7 @@
         <v/>
       </c>
       <c r="M43" s="27">
-        <f>IF(D43&lt;=0,0,I43/D43)</f>
+        <f>IF(OR(C43&lt;0.05,D43&lt;0.05),"",I43/D43)</f>
         <v/>
       </c>
     </row>
@@ -9791,7 +9800,7 @@
         <v/>
       </c>
       <c r="M44" s="27">
-        <f>IF(D44&lt;=0,0,I44/D44)</f>
+        <f>IF(OR(C44&lt;0.05,D44&lt;0.05),"",I44/D44)</f>
         <v/>
       </c>
     </row>
@@ -9844,7 +9853,7 @@
         <v/>
       </c>
       <c r="M45" s="27">
-        <f>IF(D45&lt;=0,0,I45/D45)</f>
+        <f>IF(OR(C45&lt;0.05,D45&lt;0.05),"",I45/D45)</f>
         <v/>
       </c>
     </row>
@@ -9897,7 +9906,7 @@
         <v/>
       </c>
       <c r="M46" s="27">
-        <f>IF(D46&lt;=0,0,I46/D46)</f>
+        <f>IF(OR(C46&lt;0.05,D46&lt;0.05),"",I46/D46)</f>
         <v/>
       </c>
     </row>
@@ -9950,7 +9959,7 @@
         <v/>
       </c>
       <c r="M47" s="27">
-        <f>IF(D47&lt;=0,0,I47/D47)</f>
+        <f>IF(OR(C47&lt;0.05,D47&lt;0.05),"",I47/D47)</f>
         <v/>
       </c>
     </row>
@@ -10003,7 +10012,7 @@
         <v/>
       </c>
       <c r="M48" s="27">
-        <f>IF(D48&lt;=0,0,I48/D48)</f>
+        <f>IF(OR(C48&lt;0.05,D48&lt;0.05),"",I48/D48)</f>
         <v/>
       </c>
     </row>
@@ -10056,7 +10065,7 @@
         <v/>
       </c>
       <c r="M49" s="27">
-        <f>IF(D49&lt;=0,0,I49/D49)</f>
+        <f>IF(OR(C49&lt;0.05,D49&lt;0.05),"",I49/D49)</f>
         <v/>
       </c>
     </row>
@@ -10109,7 +10118,7 @@
         <v/>
       </c>
       <c r="M50" s="27">
-        <f>IF(D50&lt;=0,0,I50/D50)</f>
+        <f>IF(OR(C50&lt;0.05,D50&lt;0.05),"",I50/D50)</f>
         <v/>
       </c>
     </row>
@@ -10162,7 +10171,7 @@
         <v/>
       </c>
       <c r="M51" s="27">
-        <f>IF(D51&lt;=0,0,I51/D51)</f>
+        <f>IF(OR(C51&lt;0.05,D51&lt;0.05),"",I51/D51)</f>
         <v/>
       </c>
     </row>
@@ -10215,7 +10224,7 @@
         <v/>
       </c>
       <c r="M52" s="27">
-        <f>IF(D52&lt;=0,0,I52/D52)</f>
+        <f>IF(OR(C52&lt;0.05,D52&lt;0.05),"",I52/D52)</f>
         <v/>
       </c>
     </row>
@@ -10268,7 +10277,7 @@
         <v/>
       </c>
       <c r="M53" s="27">
-        <f>IF(D53&lt;=0,0,I53/D53)</f>
+        <f>IF(OR(C53&lt;0.05,D53&lt;0.05),"",I53/D53)</f>
         <v/>
       </c>
     </row>
@@ -10321,7 +10330,7 @@
         <v/>
       </c>
       <c r="M54" s="27">
-        <f>IF(D54&lt;=0,0,I54/D54)</f>
+        <f>IF(OR(C54&lt;0.05,D54&lt;0.05),"",I54/D54)</f>
         <v/>
       </c>
     </row>
@@ -10374,7 +10383,7 @@
         <v/>
       </c>
       <c r="M55" s="27">
-        <f>IF(D55&lt;=0,0,I55/D55)</f>
+        <f>IF(OR(C55&lt;0.05,D55&lt;0.05),"",I55/D55)</f>
         <v/>
       </c>
     </row>
@@ -10427,7 +10436,7 @@
         <v/>
       </c>
       <c r="M56" s="27">
-        <f>IF(D56&lt;=0,0,I56/D56)</f>
+        <f>IF(OR(C56&lt;0.05,D56&lt;0.05),"",I56/D56)</f>
         <v/>
       </c>
     </row>
@@ -10480,7 +10489,7 @@
         <v/>
       </c>
       <c r="M57" s="27">
-        <f>IF(D57&lt;=0,0,I57/D57)</f>
+        <f>IF(OR(C57&lt;0.05,D57&lt;0.05),"",I57/D57)</f>
         <v/>
       </c>
     </row>
@@ -10533,7 +10542,7 @@
         <v/>
       </c>
       <c r="M58" s="27">
-        <f>IF(D58&lt;=0,0,I58/D58)</f>
+        <f>IF(OR(C58&lt;0.05,D58&lt;0.05),"",I58/D58)</f>
         <v/>
       </c>
     </row>
@@ -10586,7 +10595,7 @@
         <v/>
       </c>
       <c r="M59" s="27">
-        <f>IF(D59&lt;=0,0,I59/D59)</f>
+        <f>IF(OR(C59&lt;0.05,D59&lt;0.05),"",I59/D59)</f>
         <v/>
       </c>
     </row>
@@ -10639,7 +10648,7 @@
         <v/>
       </c>
       <c r="M60" s="27">
-        <f>IF(D60&lt;=0,0,I60/D60)</f>
+        <f>IF(OR(C60&lt;0.05,D60&lt;0.05),"",I60/D60)</f>
         <v/>
       </c>
     </row>
@@ -10692,7 +10701,7 @@
         <v/>
       </c>
       <c r="M61" s="27">
-        <f>IF(D61&lt;=0,0,I61/D61)</f>
+        <f>IF(OR(C61&lt;0.05,D61&lt;0.05),"",I61/D61)</f>
         <v/>
       </c>
     </row>
@@ -10745,7 +10754,7 @@
         <v/>
       </c>
       <c r="M62" s="27">
-        <f>IF(D62&lt;=0,0,I62/D62)</f>
+        <f>IF(OR(C62&lt;0.05,D62&lt;0.05),"",I62/D62)</f>
         <v/>
       </c>
     </row>
@@ -10798,7 +10807,7 @@
         <v/>
       </c>
       <c r="M63" s="27">
-        <f>IF(D63&lt;=0,0,I63/D63)</f>
+        <f>IF(OR(C63&lt;0.05,D63&lt;0.05),"",I63/D63)</f>
         <v/>
       </c>
     </row>
@@ -10851,7 +10860,7 @@
         <v/>
       </c>
       <c r="M64" s="27">
-        <f>IF(D64&lt;=0,0,I64/D64)</f>
+        <f>IF(OR(C64&lt;0.05,D64&lt;0.05),"",I64/D64)</f>
         <v/>
       </c>
     </row>
@@ -10904,7 +10913,7 @@
         <v/>
       </c>
       <c r="M65" s="27">
-        <f>IF(D65&lt;=0,0,I65/D65)</f>
+        <f>IF(OR(C65&lt;0.05,D65&lt;0.05),"",I65/D65)</f>
         <v/>
       </c>
     </row>
@@ -10957,7 +10966,7 @@
         <v/>
       </c>
       <c r="M66" s="27">
-        <f>IF(D66&lt;=0,0,I66/D66)</f>
+        <f>IF(OR(C66&lt;0.05,D66&lt;0.05),"",I66/D66)</f>
         <v/>
       </c>
     </row>
@@ -11010,7 +11019,7 @@
         <v/>
       </c>
       <c r="M67" s="27">
-        <f>IF(D67&lt;=0,0,I67/D67)</f>
+        <f>IF(OR(C67&lt;0.05,D67&lt;0.05),"",I67/D67)</f>
         <v/>
       </c>
     </row>
@@ -11063,7 +11072,7 @@
         <v/>
       </c>
       <c r="M68" s="27">
-        <f>IF(D68&lt;=0,0,I68/D68)</f>
+        <f>IF(OR(C68&lt;0.05,D68&lt;0.05),"",I68/D68)</f>
         <v/>
       </c>
     </row>
@@ -11116,7 +11125,7 @@
         <v/>
       </c>
       <c r="M69" s="27">
-        <f>IF(D69&lt;=0,0,I69/D69)</f>
+        <f>IF(OR(C69&lt;0.05,D69&lt;0.05),"",I69/D69)</f>
         <v/>
       </c>
     </row>
@@ -11169,7 +11178,7 @@
         <v/>
       </c>
       <c r="M70" s="27">
-        <f>IF(D70&lt;=0,0,I70/D70)</f>
+        <f>IF(OR(C70&lt;0.05,D70&lt;0.05),"",I70/D70)</f>
         <v/>
       </c>
     </row>
@@ -11222,7 +11231,7 @@
         <v/>
       </c>
       <c r="M71" s="27">
-        <f>IF(D71&lt;=0,0,I71/D71)</f>
+        <f>IF(OR(C71&lt;0.05,D71&lt;0.05),"",I71/D71)</f>
         <v/>
       </c>
     </row>
@@ -11275,7 +11284,7 @@
         <v/>
       </c>
       <c r="M72" s="27">
-        <f>IF(D72&lt;=0,0,I72/D72)</f>
+        <f>IF(OR(C72&lt;0.05,D72&lt;0.05),"",I72/D72)</f>
         <v/>
       </c>
     </row>
@@ -11328,7 +11337,7 @@
         <v/>
       </c>
       <c r="M73" s="27">
-        <f>IF(D73&lt;=0,0,I73/D73)</f>
+        <f>IF(OR(C73&lt;0.05,D73&lt;0.05),"",I73/D73)</f>
         <v/>
       </c>
     </row>
@@ -11381,7 +11390,7 @@
         <v/>
       </c>
       <c r="M74" s="27">
-        <f>IF(D74&lt;=0,0,I74/D74)</f>
+        <f>IF(OR(C74&lt;0.05,D74&lt;0.05),"",I74/D74)</f>
         <v/>
       </c>
     </row>
@@ -11434,7 +11443,7 @@
         <v/>
       </c>
       <c r="M75" s="27">
-        <f>IF(D75&lt;=0,0,I75/D75)</f>
+        <f>IF(OR(C75&lt;0.05,D75&lt;0.05),"",I75/D75)</f>
         <v/>
       </c>
     </row>
@@ -11487,7 +11496,7 @@
         <v/>
       </c>
       <c r="M76" s="27">
-        <f>IF(D76&lt;=0,0,I76/D76)</f>
+        <f>IF(OR(C76&lt;0.05,D76&lt;0.05),"",I76/D76)</f>
         <v/>
       </c>
     </row>
@@ -11540,7 +11549,7 @@
         <v/>
       </c>
       <c r="M77" s="27">
-        <f>IF(D77&lt;=0,0,I77/D77)</f>
+        <f>IF(OR(C77&lt;0.05,D77&lt;0.05),"",I77/D77)</f>
         <v/>
       </c>
     </row>
@@ -11593,7 +11602,7 @@
         <v/>
       </c>
       <c r="M78" s="27">
-        <f>IF(D78&lt;=0,0,I78/D78)</f>
+        <f>IF(OR(C78&lt;0.05,D78&lt;0.05),"",I78/D78)</f>
         <v/>
       </c>
     </row>
@@ -11646,7 +11655,7 @@
         <v/>
       </c>
       <c r="M79" s="27">
-        <f>IF(D79&lt;=0,0,I79/D79)</f>
+        <f>IF(OR(C79&lt;0.05,D79&lt;0.05),"",I79/D79)</f>
         <v/>
       </c>
     </row>
@@ -11699,7 +11708,7 @@
         <v/>
       </c>
       <c r="M80" s="27">
-        <f>IF(D80&lt;=0,0,I80/D80)</f>
+        <f>IF(OR(C80&lt;0.05,D80&lt;0.05),"",I80/D80)</f>
         <v/>
       </c>
     </row>
@@ -11752,7 +11761,7 @@
         <v/>
       </c>
       <c r="M81" s="27">
-        <f>IF(D81&lt;=0,0,I81/D81)</f>
+        <f>IF(OR(C81&lt;0.05,D81&lt;0.05),"",I81/D81)</f>
         <v/>
       </c>
     </row>
@@ -11805,7 +11814,7 @@
         <v/>
       </c>
       <c r="M82" s="27">
-        <f>IF(D82&lt;=0,0,I82/D82)</f>
+        <f>IF(OR(C82&lt;0.05,D82&lt;0.05),"",I82/D82)</f>
         <v/>
       </c>
     </row>
@@ -11858,7 +11867,7 @@
         <v/>
       </c>
       <c r="M83" s="27">
-        <f>IF(D83&lt;=0,0,I83/D83)</f>
+        <f>IF(OR(C83&lt;0.05,D83&lt;0.05),"",I83/D83)</f>
         <v/>
       </c>
     </row>
@@ -11911,7 +11920,7 @@
         <v/>
       </c>
       <c r="M84" s="27">
-        <f>IF(D84&lt;=0,0,I84/D84)</f>
+        <f>IF(OR(C84&lt;0.05,D84&lt;0.05),"",I84/D84)</f>
         <v/>
       </c>
     </row>
@@ -11964,7 +11973,7 @@
         <v/>
       </c>
       <c r="M85" s="27">
-        <f>IF(D85&lt;=0,0,I85/D85)</f>
+        <f>IF(OR(C85&lt;0.05,D85&lt;0.05),"",I85/D85)</f>
         <v/>
       </c>
     </row>
@@ -12017,7 +12026,7 @@
         <v/>
       </c>
       <c r="M86" s="27">
-        <f>IF(D86&lt;=0,0,I86/D86)</f>
+        <f>IF(OR(C86&lt;0.05,D86&lt;0.05),"",I86/D86)</f>
         <v/>
       </c>
     </row>
@@ -12070,7 +12079,7 @@
         <v/>
       </c>
       <c r="M87" s="27">
-        <f>IF(D87&lt;=0,0,I87/D87)</f>
+        <f>IF(OR(C87&lt;0.05,D87&lt;0.05),"",I87/D87)</f>
         <v/>
       </c>
     </row>
@@ -12123,7 +12132,7 @@
         <v/>
       </c>
       <c r="M88" s="27">
-        <f>IF(D88&lt;=0,0,I88/D88)</f>
+        <f>IF(OR(C88&lt;0.05,D88&lt;0.05),"",I88/D88)</f>
         <v/>
       </c>
     </row>
@@ -12176,7 +12185,7 @@
         <v/>
       </c>
       <c r="M89" s="27">
-        <f>IF(D89&lt;=0,0,I89/D89)</f>
+        <f>IF(OR(C89&lt;0.05,D89&lt;0.05),"",I89/D89)</f>
         <v/>
       </c>
     </row>
@@ -12229,7 +12238,7 @@
         <v/>
       </c>
       <c r="M90" s="27">
-        <f>IF(D90&lt;=0,0,I90/D90)</f>
+        <f>IF(OR(C90&lt;0.05,D90&lt;0.05),"",I90/D90)</f>
         <v/>
       </c>
     </row>
@@ -12282,7 +12291,7 @@
         <v/>
       </c>
       <c r="M91" s="27">
-        <f>IF(D91&lt;=0,0,I91/D91)</f>
+        <f>IF(OR(C91&lt;0.05,D91&lt;0.05),"",I91/D91)</f>
         <v/>
       </c>
     </row>
@@ -12335,7 +12344,7 @@
         <v/>
       </c>
       <c r="M92" s="27">
-        <f>IF(D92&lt;=0,0,I92/D92)</f>
+        <f>IF(OR(C92&lt;0.05,D92&lt;0.05),"",I92/D92)</f>
         <v/>
       </c>
     </row>
@@ -12388,7 +12397,7 @@
         <v/>
       </c>
       <c r="M93" s="27">
-        <f>IF(D93&lt;=0,0,I93/D93)</f>
+        <f>IF(OR(C93&lt;0.05,D93&lt;0.05),"",I93/D93)</f>
         <v/>
       </c>
     </row>
@@ -12441,7 +12450,7 @@
         <v/>
       </c>
       <c r="M94" s="27">
-        <f>IF(D94&lt;=0,0,I94/D94)</f>
+        <f>IF(OR(C94&lt;0.05,D94&lt;0.05),"",I94/D94)</f>
         <v/>
       </c>
     </row>
@@ -12494,7 +12503,7 @@
         <v/>
       </c>
       <c r="M95" s="27">
-        <f>IF(D95&lt;=0,0,I95/D95)</f>
+        <f>IF(OR(C95&lt;0.05,D95&lt;0.05),"",I95/D95)</f>
         <v/>
       </c>
     </row>
@@ -12547,7 +12556,7 @@
         <v/>
       </c>
       <c r="M96" s="27">
-        <f>IF(D96&lt;=0,0,I96/D96)</f>
+        <f>IF(OR(C96&lt;0.05,D96&lt;0.05),"",I96/D96)</f>
         <v/>
       </c>
     </row>
@@ -12600,7 +12609,7 @@
         <v/>
       </c>
       <c r="M97" s="27">
-        <f>IF(D97&lt;=0,0,I97/D97)</f>
+        <f>IF(OR(C97&lt;0.05,D97&lt;0.05),"",I97/D97)</f>
         <v/>
       </c>
     </row>
@@ -12653,7 +12662,7 @@
         <v/>
       </c>
       <c r="M98" s="27">
-        <f>IF(D98&lt;=0,0,I98/D98)</f>
+        <f>IF(OR(C98&lt;0.05,D98&lt;0.05),"",I98/D98)</f>
         <v/>
       </c>
     </row>
@@ -12706,7 +12715,7 @@
         <v/>
       </c>
       <c r="M99" s="27">
-        <f>IF(D99&lt;=0,0,I99/D99)</f>
+        <f>IF(OR(C99&lt;0.05,D99&lt;0.05),"",I99/D99)</f>
         <v/>
       </c>
     </row>
@@ -12759,7 +12768,7 @@
         <v/>
       </c>
       <c r="M100" s="27">
-        <f>IF(D100&lt;=0,0,I100/D100)</f>
+        <f>IF(OR(C100&lt;0.05,D100&lt;0.05),"",I100/D100)</f>
         <v/>
       </c>
     </row>
@@ -12812,7 +12821,7 @@
         <v/>
       </c>
       <c r="M101" s="27">
-        <f>IF(D101&lt;=0,0,I101/D101)</f>
+        <f>IF(OR(C101&lt;0.05,D101&lt;0.05),"",I101/D101)</f>
         <v/>
       </c>
     </row>
@@ -12865,7 +12874,7 @@
         <v/>
       </c>
       <c r="M102" s="27">
-        <f>IF(D102&lt;=0,0,I102/D102)</f>
+        <f>IF(OR(C102&lt;0.05,D102&lt;0.05),"",I102/D102)</f>
         <v/>
       </c>
     </row>
@@ -12918,7 +12927,7 @@
         <v/>
       </c>
       <c r="M103" s="27">
-        <f>IF(D103&lt;=0,0,I103/D103)</f>
+        <f>IF(OR(C103&lt;0.05,D103&lt;0.05),"",I103/D103)</f>
         <v/>
       </c>
     </row>
@@ -12971,7 +12980,7 @@
         <v/>
       </c>
       <c r="M104" s="27">
-        <f>IF(D104&lt;=0,0,I104/D104)</f>
+        <f>IF(OR(C104&lt;0.05,D104&lt;0.05),"",I104/D104)</f>
         <v/>
       </c>
     </row>
@@ -13024,7 +13033,7 @@
         <v/>
       </c>
       <c r="M105" s="27">
-        <f>IF(D105&lt;=0,0,I105/D105)</f>
+        <f>IF(OR(C105&lt;0.05,D105&lt;0.05),"",I105/D105)</f>
         <v/>
       </c>
     </row>
@@ -13077,7 +13086,7 @@
         <v/>
       </c>
       <c r="M106" s="27">
-        <f>IF(D106&lt;=0,0,I106/D106)</f>
+        <f>IF(OR(C106&lt;0.05,D106&lt;0.05),"",I106/D106)</f>
         <v/>
       </c>
     </row>
@@ -13130,7 +13139,7 @@
         <v/>
       </c>
       <c r="M107" s="27">
-        <f>IF(D107&lt;=0,0,I107/D107)</f>
+        <f>IF(OR(C107&lt;0.05,D107&lt;0.05),"",I107/D107)</f>
         <v/>
       </c>
     </row>
@@ -13235,7 +13244,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>V_eq_Ø900 = Qout_total/A_plein Ø900 (indicatif; si overflow, une partie du débit n'est pas dans le tuyau)</t>
+          <t>V_pipe_seul = Qout/A_plein Ø900 seulement si WSE≤crest (pas d'overflow). Si Overflow=oui → cellule vide: lire V_Ø900 et V_overflow sur Compose_900 (ne pas diviser Qout total par A_tuyau).</t>
         </is>
       </c>
     </row>
@@ -13277,7 +13286,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>V_eq_Ø900 (m/s)</t>
+          <t>V_pipe_seul (m/s)</t>
         </is>
       </c>
     </row>
@@ -13310,7 +13319,7 @@
         </is>
       </c>
       <c r="H12" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D12/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C12&gt;$B$6),"",D12/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13344,7 +13353,7 @@
         <v/>
       </c>
       <c r="H13" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D13/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C13&gt;$B$6),"",D13/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13378,7 +13387,7 @@
         <v/>
       </c>
       <c r="H14" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D14/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C14&gt;$B$6),"",D14/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13412,7 +13421,7 @@
         <v/>
       </c>
       <c r="H15" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D15/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C15&gt;$B$6),"",D15/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13446,7 +13455,7 @@
         <v/>
       </c>
       <c r="H16" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D16/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C16&gt;$B$6),"",D16/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13480,7 +13489,7 @@
         <v/>
       </c>
       <c r="H17" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D17/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C17&gt;$B$6),"",D17/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13514,7 +13523,7 @@
         <v/>
       </c>
       <c r="H18" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D18/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C18&gt;$B$6),"",D18/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13548,7 +13557,7 @@
         <v/>
       </c>
       <c r="H19" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D19/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C19&gt;$B$6),"",D19/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13582,7 +13591,7 @@
         <v/>
       </c>
       <c r="H20" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D20/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C20&gt;$B$6),"",D20/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13616,7 +13625,7 @@
         <v/>
       </c>
       <c r="H21" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D21/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C21&gt;$B$6),"",D21/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13650,7 +13659,7 @@
         <v/>
       </c>
       <c r="H22" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D22/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C22&gt;$B$6),"",D22/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13684,7 +13693,7 @@
         <v/>
       </c>
       <c r="H23" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D23/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C23&gt;$B$6),"",D23/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>
@@ -13718,7 +13727,7 @@
         <v/>
       </c>
       <c r="H24" s="27">
-        <f>IF(Parametres!$C$87&lt;=0,0,D24/Parametres!$C$87)</f>
+        <f>IF(OR(Parametres!$C$87&lt;=0,C24&gt;$B$6),"",D24/Parametres!$C$87)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Ø900 Manning n to 0.022 for TOG (not concrete)
Q_plein drops from ~1.67 to ~0.99 m³/s; Parametres and Courbe_QH_900 updated in Deux_Zones and Ponceau_900.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Deux_Zones_1500_900_1200.xlsx
@@ -1830,7 +1830,7 @@
         <v>0.008489634748272452</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>1.668</v>
+        <v>0.986</v>
       </c>
     </row>
     <row r="7">
@@ -1874,7 +1874,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Capacité Ø900 — Manning pleine section (n = 0,013)</t>
+          <t>Capacité Ø900 — Manning pleine section (TOG n = 0,022)</t>
         </is>
       </c>
     </row>
@@ -1885,11 +1885,11 @@
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>0.013</v>
+        <v>0.022</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fourni (béton typique ~0,012–0,015)</t>
+          <t>TOG (tuyau ondulé galvanisé) n=0,022 — pas béton</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (n=0,013).</t>
+          <t>• Méthode A: Qout fixe = Q_plein Manning Ø900 (TOG n=0,022).</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   A) Q_plein Manning (n=0.013) ≈ 1.668 m³/s → Méthode A (constant).</t>
+          <t xml:space="preserve">   A) Q_plein Manning (TOG n=0.022) ≈ 0.986 m³/s → Méthode A (constant).</t>
         </is>
       </c>
     </row>
@@ -5115,11 +5115,11 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>0.013</v>
+        <v>0.022</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>béton typ. 0.012–0.015</t>
+          <t>TOG n=0,022 (ondulé galvanisé)</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">

</xml_diff>